<commit_message>
fix : add git ignore to assets
</commit_message>
<xml_diff>
--- a/assets/format/downladBase/3A.xlsx
+++ b/assets/format/downladBase/3A.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\siisd-ci-3\assets\format\downladBase\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SIISD-CI3\assets\format\downladBase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6478FE2-FA28-4131-AC40-C1D4E221C668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3439837F-4252-4A0E-806E-2C56BEA7D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1850D593-1557-4F5D-BDE3-BC3E75414898}"/>
   </bookViews>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>No</t>
   </si>
@@ -52,6 +43,15 @@
   </si>
   <si>
     <t>Alokasi APBD OP Irigasi</t>
+  </si>
+  <si>
+    <t>Alokasi APBD DAK OP Irigasi</t>
+  </si>
+  <si>
+    <t>Jumlah Orang</t>
+  </si>
+  <si>
+    <t>Kebutuhan Orang</t>
   </si>
 </sst>
 </file>
@@ -462,81 +462,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{293543DF-57F7-41C8-8A38-7EA09EA38864}">
-  <dimension ref="A2:F5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="14.77734375" customWidth="1"/>
-    <col min="9" max="9" width="19.77734375" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="15" max="15" width="10.109375" customWidth="1"/>
-    <col min="16" max="17" width="11.109375" customWidth="1"/>
-    <col min="20" max="21" width="11" customWidth="1"/>
-    <col min="22" max="22" width="10.21875" customWidth="1"/>
-    <col min="25" max="25" width="12.109375" customWidth="1"/>
-    <col min="26" max="27" width="11.77734375" customWidth="1"/>
-    <col min="30" max="30" width="11.5546875" customWidth="1"/>
-    <col min="31" max="31" width="12" customWidth="1"/>
-    <col min="32" max="32" width="10.88671875" customWidth="1"/>
-    <col min="35" max="35" width="12.6640625" customWidth="1"/>
-    <col min="36" max="36" width="12" customWidth="1"/>
-    <col min="37" max="37" width="11.44140625" customWidth="1"/>
-    <col min="38" max="38" width="14.88671875" customWidth="1"/>
-    <col min="39" max="39" width="14.5546875" customWidth="1"/>
-    <col min="40" max="40" width="14" customWidth="1"/>
-    <col min="41" max="41" width="16.77734375" customWidth="1"/>
-    <col min="42" max="42" width="11.21875" customWidth="1"/>
-    <col min="43" max="43" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" customWidth="1"/>
+    <col min="10" max="11" width="11.109375" customWidth="1"/>
+    <col min="14" max="15" width="11" customWidth="1"/>
+    <col min="16" max="16" width="10.21875" customWidth="1"/>
+    <col min="19" max="19" width="12.109375" customWidth="1"/>
+    <col min="20" max="21" width="11.77734375" customWidth="1"/>
+    <col min="24" max="24" width="11.5546875" customWidth="1"/>
+    <col min="25" max="25" width="12" customWidth="1"/>
+    <col min="26" max="26" width="10.88671875" customWidth="1"/>
+    <col min="29" max="29" width="12.6640625" customWidth="1"/>
+    <col min="30" max="30" width="12" customWidth="1"/>
+    <col min="31" max="31" width="11.44140625" customWidth="1"/>
+    <col min="32" max="32" width="14.88671875" customWidth="1"/>
+    <col min="33" max="33" width="14.5546875" customWidth="1"/>
+    <col min="34" max="34" width="14" customWidth="1"/>
+    <col min="35" max="35" width="16.77734375" customWidth="1"/>
+    <col min="36" max="36" width="11.21875" customWidth="1"/>
+    <col min="37" max="37" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:9" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="2" spans="1:9" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B2" s="2">
         <v>2</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C2" s="2">
         <v>3</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D2" s="2">
         <v>4</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E2" s="2">
         <v>5</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F2" s="2">
         <v>6</v>
       </c>
+      <c r="G2" s="2">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2">
+        <v>8</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:9" ht="19.2" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>